<commit_message>
feat(proposal): migrate 56A0TXN draft artifacts and chapter data flow
Rebase local proposal workflow changes onto latest feature_new, including chapter persistence updates, generated 56A0TXN artifacts relocation, and proposal UI chapter wiring needed for draft/save/release alignment.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/projects/56A0TXN/早期介入/交付预案/解析结果/预案草稿/2.设备配置信息.xlsx
+++ b/data/projects/56A0TXN/早期介入/交付预案/解析结果/预案草稿/2.设备配置信息.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U6"/>
+  <dimension ref="A1:R6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -507,21 +507,6 @@
           <t>设备角色</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>sourceFile</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>categoryName</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>pbiProductName</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -539,7 +524,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>CloudEngine 16800 V300R023C00SPC500</t>
+          <t>CloudEngine 16800 V300</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -594,21 +579,6 @@
       <c r="R2" t="inlineStr">
         <is>
           <t>交换机</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>京东科技网络设备_64pcsCE16800-X16_拆分_设备及服务_0X00Hc00847542202511200002_不含价格.normalized.json</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>CloudEngine 16800 &amp; XH16800 核心交换机</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>CloudEngine 16800</t>
         </is>
       </c>
     </row>
@@ -628,7 +598,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>CloudEngine 9800 V300R024C00</t>
+          <t>CloudEngine 9800 V200R025C00</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -683,21 +653,6 @@
       <c r="R3" t="inlineStr">
         <is>
           <t>交换机</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>JXX项目网络设备_76pcsCE9866_拆分_设备及服务_0X00Hc00847542202511200004_不含价格.normalized.json</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>CloudEngine 9800 &amp; XH9000 TOR 交换机</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>CloudEngine 9800</t>
         </is>
       </c>
     </row>
@@ -750,21 +705,6 @@
           <t>交换机</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
-        <is>
-          <t>京东科技网络设备_64pcsCE16800-X16_拆分_设备及服务_0X00Hc00847542202511200002_不含价格.normalized.json</t>
-        </is>
-      </c>
-      <c r="T4" t="inlineStr">
-        <is>
-          <t>CloudEngine 16800 &amp; XH16800 核心交换机</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>CloudEngine XH16800</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -815,21 +755,6 @@
           <t>交换机</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
-        <is>
-          <t>JXX项目网络设备_76pcsCE9866_拆分_设备及服务_0X00Hc00847542202511200004_不含价格.normalized.json</t>
-        </is>
-      </c>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>CloudEngine 9800 &amp; XH9000 TOR 交换机</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>CloudEngine XH9000</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -847,7 +772,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Atlas 900 A3 SuperPoD 1.0.T31</t>
+          <t>Atlas 900 A3 SuperPoD 1.0.T25</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -902,21 +827,6 @@
       <c r="R6" t="inlineStr">
         <is>
           <t>智算服务器</t>
-        </is>
-      </c>
-      <c r="S6" t="inlineStr">
-        <is>
-          <t>JXX项目2025昇腾超节点下单-三期-1-1_0000Hw00478677202512170036_不含价格-POD01.normalized.json;JXX项目2025昇腾超节点下单-三期-1-2_0000Hw00478677202512170020_不含价格-POD02.normalized.json;JXX项目2025昇腾超节点下单-三期-1-3_0000Hw00478677202512170022_不含价格-POD03.normalized.json;JXX项目2025昇腾超节点下单-三期-1-4_0000Hw00478677202512170024_不含价格-POD04.normalized.json;JXX项目2025昇腾超节点下单-三期-2-1_0000Hw00478677202512170026_不含价格-POD05.normalized.json;JXX项目2025昇腾超节点下单-三期-2-2_0000Hw00478677202512170028_不含价格-POD06.normalized.json;JXX项目2025昇腾超节点下单-三期-2-3_0000Hw00478677202512170030_不含价格-POD07.normalized.json;JXX项目2025昇腾超节点下单-三期-2-4_0000Hw00478677202512170032_不含价格-POD08.normalized.json;JXX项目2025昇腾超节点下单-三期-2-5_0000Hw00478677202512170034_不含价格-POD09.normalized.json</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr">
-        <is>
-          <t>Atlas 900 A3 SuperPoD</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>Atlas 900 A3 SuperPoD</t>
         </is>
       </c>
     </row>

</xml_diff>